<commit_message>
Remove obsolete Firebase source code files causing build errors
</commit_message>
<xml_diff>
--- a/Vectra Staffing LLC Employee Directory.xlsx
+++ b/Vectra Staffing LLC Employee Directory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\ERP-System-Production\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91447CF9-4225-4477-9C0D-FF7906C3D1B6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4996793A-A5B2-49ED-99E3-9A5E16A171FE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="19422" windowHeight="10302" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="137">
   <si>
     <t>Employee joining, designation, and contact records | Updated for 2025–2026</t>
   </si>
@@ -428,6 +428,9 @@
   </si>
   <si>
     <t>Updated Week 3</t>
+  </si>
+  <si>
+    <t>BRD not sent</t>
   </si>
 </sst>
 </file>
@@ -720,17 +723,6 @@
   <dxfs count="12">
     <dxf>
       <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
@@ -911,6 +903,17 @@
         <scheme val="major"/>
       </font>
     </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -925,18 +928,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="EmployeeDirectoryWithDesignation" displayName="EmployeeDirectoryWithDesignation" ref="A5:J38" dataDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="EmployeeDirectoryWithDesignation" displayName="EmployeeDirectoryWithDesignation" ref="A5:J38" dataDxfId="10">
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Sr. No." dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Date of Joining" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Employee Name" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Designation" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Personal Email ID" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Official Email ID" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{2E3810A5-C9F7-49A1-AEC2-94158935767D}" name="Column1" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{B81BBC40-737D-455E-BBC1-509E40D3F7D8}" name="Column2" dataDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{31800684-A15C-4EDC-9F08-3D0F7FE50F4F}" name="Column 3" dataDxfId="2"/>
-    <tableColumn id="10" xr3:uid="{95819C09-FC15-4B97-8E78-01BF41FCFA5C}" name="Column 4" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Sr. No." dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Date of Joining" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Employee Name" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Designation" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Personal Email ID" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Official Email ID" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{2E3810A5-C9F7-49A1-AEC2-94158935767D}" name="Column1" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{B81BBC40-737D-455E-BBC1-509E40D3F7D8}" name="Column2" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{31800684-A15C-4EDC-9F08-3D0F7FE50F4F}" name="Column 3" dataDxfId="1"/>
+    <tableColumn id="10" xr3:uid="{95819C09-FC15-4B97-8E78-01BF41FCFA5C}" name="Column 4" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1463,7 +1466,9 @@
       <c r="I16" s="24" t="s">
         <v>133</v>
       </c>
-      <c r="J16" s="24"/>
+      <c r="J16" s="24" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="17" spans="1:10" ht="14.4">
       <c r="A17" s="6">
@@ -1493,7 +1498,9 @@
       <c r="I17" s="24" t="s">
         <v>133</v>
       </c>
-      <c r="J17" s="24"/>
+      <c r="J17" s="24" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="18" spans="1:10" ht="14.4">
       <c r="A18" s="10">
@@ -1521,7 +1528,9 @@
         <v>122</v>
       </c>
       <c r="I18" s="24"/>
-      <c r="J18" s="24"/>
+      <c r="J18" s="24" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="19" spans="1:10" ht="14.4">
       <c r="A19" s="6"/>
@@ -1589,7 +1598,9 @@
       <c r="I21" s="24" t="s">
         <v>133</v>
       </c>
-      <c r="J21" s="24"/>
+      <c r="J21" s="24" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="22" spans="1:10" ht="14.4">
       <c r="A22" s="10">
@@ -1619,7 +1630,9 @@
       <c r="I22" s="24" t="s">
         <v>133</v>
       </c>
-      <c r="J22" s="24"/>
+      <c r="J22" s="24" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="23" spans="1:10" ht="14.4">
       <c r="A23" s="6">
@@ -1649,7 +1662,9 @@
       <c r="I23" s="24" t="s">
         <v>133</v>
       </c>
-      <c r="J23" s="24"/>
+      <c r="J23" s="24" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="24" spans="1:10" ht="14.4">
       <c r="A24" s="10"/>
@@ -1691,7 +1706,9 @@
       <c r="I25" s="24" t="s">
         <v>133</v>
       </c>
-      <c r="J25" s="24"/>
+      <c r="J25" s="24" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="26" spans="1:10" ht="14.4">
       <c r="A26" s="10">
@@ -1721,7 +1738,9 @@
       <c r="I26" s="24" t="s">
         <v>133</v>
       </c>
-      <c r="J26" s="24"/>
+      <c r="J26" s="24" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="27" spans="1:10" ht="14.4">
       <c r="A27" s="6">
@@ -1751,7 +1770,9 @@
       <c r="I27" s="24" t="s">
         <v>133</v>
       </c>
-      <c r="J27" s="24"/>
+      <c r="J27" s="24" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="28" spans="1:10" ht="14.4">
       <c r="A28" s="10"/>
@@ -2028,7 +2049,7 @@
     <mergeCell ref="A3:F3"/>
   </mergeCells>
   <conditionalFormatting sqref="D6:D20 D23 D25:D38">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="11" priority="1">
       <formula>D6="Not Available"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>